<commit_message>
data: add verified urethral prostate paper
</commit_message>
<xml_diff>
--- a/db/cellxgene/pns_papers_summary.xlsx
+++ b/db/cellxgene/pns_papers_summary.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rce97d36e6e7041e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8be27231ccfb4fa8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3851,10 +3851,11 @@
           <x:t xml:space="preserve">10x 3' v2</x:t>
         </x:is>
       </x:c>
-      <x:c r="I68" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">N</x:t>
-        </x:is>
+      <x:c r="I68" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>D:\OneDrive\Desktop\组\db\cellxgene\cellxgene_filtered\downloads\PMID_32497356_Urethral luminal epithelia are castration-insensitive cells of the proximal prostate.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="69">

</xml_diff>

<commit_message>
data: add verified kidney zonation paper
</commit_message>
<xml_diff>
--- a/db/cellxgene/pns_papers_summary.xlsx
+++ b/db/cellxgene/pns_papers_summary.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8be27231ccfb4fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R319b36164256478c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3951,15 +3951,11 @@
           <x:t xml:space="preserve">10x 3' v2</x:t>
         </x:is>
       </x:c>
-      <x:c r="I70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Y</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D:\OneDrive\Desktop\组\db\cellxgene\cellxgene_filtered\downloads\PMID_31604275_Spatiotemporal immune zonation of the human kidney..pdf</x:t>
-        </x:is>
+      <x:c r="I70" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>D:\OneDrive\Desktop\组\db\cellxgene\cellxgene_filtered\downloads\PMID_31604275_Spatiotemporal immune zonation of the human kidney.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="71">

</xml_diff>